<commit_message>
fix: preserve inventory template compatibility
</commit_message>
<xml_diff>
--- a/outputs/inventory_import_template/과거_재고_간단_입력_양식.xlsx
+++ b/outputs/inventory_import_template/과거_재고_간단_입력_양식.xlsx
@@ -491,6 +491,9 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetPr>
+    <x:pageSetUpPr fitToPage="1"/>
+  </x:sheetPr>
   <x:sheetFormatPr defaultRowHeight="20.100000381469727"/>
   <x:sheetData>
     <x:row r="1" ht="20.100000381469727" customHeight="1">
@@ -519,11 +522,15 @@
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:pageSetup fitToHeight="0" orientation="landscape"/>
 </x:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetPr>
+    <x:pageSetUpPr fitToPage="1"/>
+  </x:sheetPr>
   <x:sheetFormatPr defaultRowHeight="20.100000381469727"/>
   <x:cols>
     <x:col min="1" max="1" width="16" customWidth="1"/>
@@ -613,11 +620,15 @@
     <x:mergeCell ref="A11:F11"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:pageSetup fitToHeight="0" orientation="landscape"/>
 </x:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetPr>
+    <x:pageSetUpPr fitToPage="1"/>
+  </x:sheetPr>
   <x:sheetFormatPr defaultRowHeight="20.100000381469727"/>
   <x:cols>
     <x:col min="1" max="1" width="14" style="4" customWidth="1"/>
@@ -30742,22 +30753,26 @@
     <x:dataValidation type="date" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorTitle="날짜 확인" error="날짜는 yyyy-mm-dd 형식으로 입력해 주세요." sqref="A4:A2004">
       <x:formula1>43830.625</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" errorStyle="stop" showErrorMessage="1" errorTitle="입력 확인" error="목록에서 선택해 주세요." sqref="E4:E2004">
+    <x:dataValidation allowBlank="1" type="list" errorStyle="stop" showErrorMessage="1" errorTitle="입력 확인" error="목록에서 선택해 주세요." sqref="E4:E2004">
       <x:formula1>'선택목록'!$A$2:$A$3</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="custom" errorStyle="stop" showErrorMessage="1" errorTitle="수량 확인" error="0 이상의 수량을 소수점 첫째 자리까지 입력해 주세요." sqref="F4:F2004">
+    <x:dataValidation allowBlank="1" type="custom" errorStyle="stop" showErrorMessage="1" errorTitle="수량 확인" error="0 이상의 수량을 소수점 첫째 자리까지 입력해 주세요." sqref="F4:F2004">
       <x:formula1>OR(F4="",AND(ISNUMBER(F4),F4&gt;=0,ROUND(F4,1)=F4))</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="whole" errorStyle="stop" operator="greaterThanOrEqual" showErrorMessage="1" errorTitle="숫자 확인" error="0 이상의 정수만 입력해 주세요." sqref="G4:G2004">
+    <x:dataValidation allowBlank="1" type="whole" errorStyle="stop" operator="greaterThanOrEqual" showErrorMessage="1" errorTitle="숫자 확인" error="0 이상의 정수만 입력해 주세요." sqref="G4:G2004">
       <x:formula1>0</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:pageSetup fitToHeight="0" orientation="landscape"/>
 </x:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetPr>
+    <x:pageSetUpPr fitToPage="1"/>
+  </x:sheetPr>
   <x:sheetFormatPr defaultRowHeight="20.100000381469727"/>
   <x:cols>
     <x:col min="1" max="1" width="14" style="4" customWidth="1"/>
@@ -43864,13 +43879,14 @@
     <x:dataValidation type="date" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorTitle="날짜 확인" error="날짜는 yyyy-mm-dd 형식으로 입력해 주세요." sqref="A4:A1004 E4:E1004">
       <x:formula1>43830.625</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="whole" errorStyle="stop" operator="greaterThanOrEqual" showErrorMessage="1" errorTitle="숫자 확인" error="0 이상의 정수만 입력해 주세요." sqref="F4:F1004">
+    <x:dataValidation allowBlank="1" type="whole" errorStyle="stop" operator="greaterThanOrEqual" showErrorMessage="1" errorTitle="숫자 확인" error="0 이상의 정수만 입력해 주세요." sqref="F4:F1004">
       <x:formula1>0</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="custom" errorStyle="stop" showErrorMessage="1" errorTitle="수량 확인" error="0 이상의 수량을 소수점 첫째 자리까지 입력해 주세요." sqref="G4:G1004">
+    <x:dataValidation allowBlank="1" type="custom" errorStyle="stop" showErrorMessage="1" errorTitle="수량 확인" error="0 이상의 수량을 소수점 첫째 자리까지 입력해 주세요." sqref="G4:G1004">
       <x:formula1>OR(G4="",AND(ISNUMBER(G4),G4&gt;=0,ROUND(G4,1)=G4))</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:pageSetup fitToHeight="0" orientation="landscape"/>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
fix: preserve opening template blank validation
</commit_message>
<xml_diff>
--- a/outputs/inventory_import_template/과거_재고_간단_입력_양식.xlsx
+++ b/outputs/inventory_import_template/과거_재고_간단_입력_양식.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="선택목록" sheetId="1" r:id="R938cb4334f444f88"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="작성방법" sheetId="2" r:id="Rcfd9f65656234a7c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="재고입력" sheetId="3" r:id="R92a8a8cf981b49eb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="입고별잔량_선택" sheetId="4" r:id="Rdfbfa8f38b6c4e62"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="선택목록" sheetId="1" r:id="R4f2dbf7942464c0a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="작성방법" sheetId="2" r:id="Ra5097b4867404b31"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="재고입력" sheetId="3" r:id="R7643fe7393424466"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="입고별잔량_선택" sheetId="4" r:id="R1a1d2123f4754e66"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -32418,7 +32418,7 @@
     <x:dataValidation type="date" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorTitle="날짜 확인" error="날짜는 yyyy-mm-dd 형식으로 입력해 주세요." sqref="A4:A2004">
       <x:formula1>43830.625</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" errorStyle="stop" showErrorMessage="1" errorTitle="입력 확인" error="목록에서 선택해 주세요." sqref="E4:E72">
+    <x:dataValidation type="list" errorStyle="stop" allowBlank="1" showErrorMessage="1" errorTitle="입력 확인" error="목록에서 선택해 주세요." sqref="E4:E72">
       <x:formula1>선택목록!$A$2:$A$3</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="custom" errorStyle="stop" showErrorMessage="1" errorTitle="수량 확인" error="0 이상의 수량을 소수점 둘째 자리까지 입력해 주세요." sqref="F4:F2004">

</xml_diff>